<commit_message>
Publish Moscow_2014_WCH, OklahomaCity_2014_MAR, Szeged_2014_JWCH, Szeged_2014_WC
</commit_message>
<xml_diff>
--- a/events/OklahomaCity_2014_MAR/OklahomaCity_2014_MAR_Results.xlsx
+++ b/events/OklahomaCity_2014_MAR/OklahomaCity_2014_MAR_Results.xlsx
@@ -7094,6 +7094,11 @@
           <t>56154</t>
         </is>
       </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>94098</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -16632,7 +16637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D175"/>
+  <dimension ref="A1:D176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20485,6 +20490,28 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>94098</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Jean</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>VAN DER WESTHUIZEN</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>